<commit_message>
Leads: 2026-09-25 00:07 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://bufordplumbing.net/</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>info@bufordplumbing.net</t>
@@ -554,6 +553,66 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nashua, NH  Residential Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>scottsroofing.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.scottsroofing.com/index.php/nashua-residential-roofing-contractor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Gallery Financing</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>mymail@mailservice.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>555-555-5555</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Nashua NH</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>residential roofing company Nashua NH</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 00:10 UTC (cycle 176)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -618,6 +618,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Alexandria Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>alexandria-hvac.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.alexandria-hvac.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Services Call</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@alexandria-hvac.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(703) 202-6140</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>heating and cooling company Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 00:20 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AC Installation in Lewiston, ME | RG Mechanical</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>rgmechanicalhomeservices.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://rgmechanicalhomeservices.com/cooling/central-air/lewiston-me</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Big Company</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>rgmechanicalme@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(207) 441-5820</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Lewiston ME</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>AC installation Lewiston ME</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 00:37 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>G&amp;J Roofing Corp of South Florida</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>gjroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://gjroofingfl.com/service-areas/hollywood/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Roofing Corp</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>gjroofingfl@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>954-729-0590</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 00:42 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Equinox Roofing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>equinox-roofing.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://equinox-roofing.com/service-areas/alameda-county/fremont/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Roof Inspection</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>equinoxroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(800) 880-6020</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>residential roofing company Fremont CA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 00:46 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Capitan's</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>capitansrestoration.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.capitansrestoration.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Insurance Claims</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(216) 350-7979</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>96</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roof repair company Akron OH</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:32 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alliance Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>alliancehvac.tech</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://alliancehvac.tech/cincinnati-oh/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Plan Cincinnati</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>alliancehvac1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>859) 551-0056</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>heating and cooling company Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:33 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,62 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Metal Roofing Alpharetta</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rackleyroofingandsupplyga.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://rackleyroofingandsupplyga.com/areas-of-service/alpharetta-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>rackley03@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(770) 771-8802</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:34 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -999,7 +999,6 @@
           <t>https://rackleyroofingandsupplyga.com/areas-of-service/alpharetta-metal-roofing/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>rackley03@gmail.com</t>
@@ -1029,6 +1028,62 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Glacier Roof Renew</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>glacierroofrenew.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://glacierroofrenew.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>matthewwwheeler@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(512) 577-3895</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roof replacement Missoula MT</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:37 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1054,7 +1054,6 @@
           <t>https://glacierroofrenew.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>matthewwwheeler@gmail.com</t>
@@ -1084,6 +1083,122 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tytum</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>tytum.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://tytum.com/services/heating-and-air/air-conditioning</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>contact@tytum.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(619) 349-4397</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>air conditioning repair San Diego CA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Roof Repair in Dallas, TX | Same-Day Local Service</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>roofingprosdallastx.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://roofingprosdallastx.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@roofingprosdallastx.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(469) 746-9771</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roof repair company Dallas TX</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:39 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1109,7 +1109,6 @@
           <t>https://tytum.com/services/heating-and-air/air-conditioning</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>contact@tytum.com</t>
@@ -1199,6 +1198,66 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Reynolds Heat N Air</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>reynoldsheatnair.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://reynoldsheatnair.com/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Reynolds Heat</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>scott@reynoldsheatnair.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(972) 725-4105</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>heat pump installation Dallas TX</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:40 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1263,6 +1263,62 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SN Heating and AC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>snheatingandac.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.snheatingandac.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@snheatingandac.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(209) 684-6628</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>HVAC contractor Stockton CA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:43 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1284,6 @@
           <t>https://www.snheatingandac.com/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@snheatingandac.com</t>
@@ -1314,6 +1313,62 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation Services | Kansas City Metro Area</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>mosheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.mosheatingandcooling.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>mosheatingandair@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(913) 213-1536</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Kansas City MO</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>heat pump installation Kansas City MO</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:52 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1339,7 +1339,6 @@
           <t>https://www.mosheatingandcooling.com/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>mosheatingandair@yahoo.com</t>
@@ -1369,6 +1368,62 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Carson City</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nevadaplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://nevadaplumbingservice.com/locations/carson-city-nv/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@nevadaplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(702) 268-2148</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Carson City NV</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>drain cleaning service Carson City NV</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 13:55 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1394,7 +1394,6 @@
           <t>https://nevadaplumbingservice.com/locations/carson-city-nv/drain-cleaning</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>info@nevadaplumbingservice.com</t>
@@ -1424,6 +1423,66 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>A&amp;H Roofing &amp; Contracting, LLC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ahroofingcontracting.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.ahroofingcontracting.com/services/roofing-contractor/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Roofing And</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>admin@ahroofingcontracting.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(918) 550-9886</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roof replacement Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 14:02 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1488,6 +1488,66 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rest Assured HVAC â Your Local Family Owned &amp; Operated HVAC Contractor serving</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>restassuredhvac.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://restassuredhvac.com/services/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Thanks Fred</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@restassuredhvac.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(847) 224-2420</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>air conditioning repair Elgin IL</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 14:12 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1548,6 +1548,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tapped Out Plumbing and Backflow</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>tappedoutplumbingandbackflow.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://tappedoutplumbingandbackflow.com/sewer-services/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>North Texas</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>office@tappedoutplumbingandbackflow.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>469-826-3610</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>sewer repair Denton TX</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 14:49 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1608,6 +1608,122 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Farrell's Heating and air Conditioning</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>farrellheating.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.farrellheating.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@farrellheating.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(712) 233-3005</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Sioux City IA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sioux City IA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CW Suter Services</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>cwsuter.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://cwsuter.com/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Owned As</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>lmoore@cwsuter.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>712.252.3007</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Sioux City IA</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sioux City IA</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 14:55 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1629,7 +1629,6 @@
           <t>https://www.farrellheating.com/</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>info@farrellheating.com</t>
@@ -1719,6 +1718,66 @@
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Icon Roofing Group</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>iconroofinggroup.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.iconroofinggroup.com/kissimmee-roofing-contractor/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Insurance Claims</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info@iconroofinggroup.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(407) 476-9166</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roofing contractor Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 14:56 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1783,6 +1783,62 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thorpe Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>southlandair.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://southlandair.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@southlandach.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(504) 469-3132</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>AC installation New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 14:58 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1804,7 +1804,6 @@
           <t>https://southlandair.com/</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>info@southlandach.com</t>
@@ -1834,6 +1833,66 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Plano Roof Guys | #1 Roofing Contractor in Plano, TX – Free Inspections</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>planoroofguys.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://planoroofguys.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Why Plano</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>info@planoroofguys.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(469) 306-0506</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>roofing contractor Plano TX</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 15:24 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1898,6 +1898,66 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cliffrose Roofing Co.</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>adojo.net</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.adojo.net/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>St George</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>hello@cliffroseroofing.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(435) 555-0142</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St George UT</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 15:27 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1958,6 +1958,62 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Reliance Mechanical</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>relyonreliance.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://relyonreliance.com/plumbing/water-heater</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>service@relyonreliance.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(228) 819-7473</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Gulfport MS</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>90</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>water heater repair Gulfport MS</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 15:46 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1979,7 +1979,6 @@
           <t>https://relyonreliance.com/plumbing/water-heater</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>service@relyonreliance.com</t>
@@ -2009,6 +2008,126 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Atlas AC Repair, LLC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>atlasacrepair.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://atlasacrepair.com/service-areas/san-antonio-tx/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Transparency Transparency</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>info@atlasacrepair.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(210) 549-9550</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>heat pump installation San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Wright Home Services</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>wrightac.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.wrightac.com/heating/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Wright Home</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>info@wrightac.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(210) 599-7000</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>heat pump installation San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 15:50 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2133,6 +2133,66 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Three Guys Master Tradesmen</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3gmt.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://3gmt.com/hvac/services/ac-install/pinellas-county/st-petersburg/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Snell Is</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@3gmt.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(727) 201-1100</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>94</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>AC installation St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 15:51 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2193,6 +2193,62 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AC Repair Gilbert | East Valley Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>eastvalleyacs.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.eastvalleyacs.com/ac-repair-gilbert</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>contact@eastvalleyacs.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>602-869-4275</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>98</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>air conditioning repair Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 15:54 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2214,7 +2214,6 @@
           <t>https://www.eastvalleyacs.com/ac-repair-gilbert</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>contact@eastvalleyacs.com</t>
@@ -2244,6 +2243,126 @@
         </is>
       </c>
       <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Cool Aid Air Conditioning and Refrigeration</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1800coolaid.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://1800coolaid.com/san-jose-hvac-refrigeration/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Call Now</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>info@1800coolaid.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>800-266-5243</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>San Jose CA</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>heat pump installation San Jose CA</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Air Care Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>aircareheatandcool.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://aircareheatandcool.com/services/heat-pumps/installation</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Project View</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>info@hvac-aircare.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>408.317.2950</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>San Jose CA</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>heat pump installation San Jose CA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:10 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2368,6 +2368,66 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Richardson, TX - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>richardsonhvacpro.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://richardsonhvacpro.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Coit Rd</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>info@richardsonhvacpro.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(214) 833-5592</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>100</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>heating and cooling company Richardson TX</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:13 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2428,6 +2428,62 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MBD Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>mbdhvac.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://mbdhvac.com/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>office@mbdhvac.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(732) 880-7999</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>heating and cooling company Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:25 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2449,7 +2449,6 @@
           <t>https://mbdhvac.com/</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>office@mbdhvac.com</t>
@@ -2479,6 +2478,66 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>APE Roofing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>aperoofing.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://aperoofing.com/fort-collins/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Founder Grounded</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>customerservice@aperoofing.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(720) 310-0050</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>roof replacement Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:29 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2543,6 +2543,66 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Providence RI | F.G. Lees &amp; Son</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>fglees.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.fglees.com/plumbing-services/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Makers Require</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>accounting@fglees.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(401) 421-1358</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Providence RI</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>drain cleaning service Providence RI</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:37 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2603,6 +2603,62 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Rhino Commercial Roofing</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>rhinocommercialroofers.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://rhinocommercialroofers.com/metal-roofing-st-petersburg-fl/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>rhinoroofingfl@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>813-336-5415</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>98</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:41 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2624,7 +2624,6 @@
           <t>https://rhinocommercialroofers.com/metal-roofing-st-petersburg-fl/</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>rhinoroofingfl@yahoo.com</t>
@@ -2654,6 +2653,62 @@
         </is>
       </c>
       <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Guaranteed Mechanical Service Inc.</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>guaranteedmechanical.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://guaranteedmechanical.com/hvac/aurora-il/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>tony@guaranteedmechanical.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>630.692.3901</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>heat pump installation Aurora IL</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:43 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2679,7 +2679,6 @@
           <t>https://guaranteedmechanical.com/hvac/aurora-il/heat-pump-installation/</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>tony@guaranteedmechanical.com</t>
@@ -2709,6 +2708,126 @@
         </is>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Plumbing Ankeny</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>plumbingankeny.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://plumbingankeny.com/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Speed At</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>service@plumbingankeny.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(831) 290-4327</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>100</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>emergency plumber Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Chad Baker Drain Cleaning Plumbing HVAC</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>chadbaker.net</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.chadbaker.net/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Local Racing</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>admin@chadbaker.net</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>717-599-8044</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>82</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>emergency plumber Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 16:59 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2833,6 +2833,126 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Martin Moran Roofing</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>mmroofs.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://mmroofs.com/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Kiddar Capital</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>info@mmroofs.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(209) 315-5553</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Modesto CA</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>residential roofing company Modesto CA</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Native Roofing and Solar</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>nativecoso.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.nativecoso.com/springfield</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Native Roofing</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>info@nativecoso.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(855) 755-5400</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Springfield IL</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>86</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>roofing contractor Springfield IL</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:06 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2953,6 +2953,66 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Salem Apex Plumbing</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>apexplumbersalem.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://apexplumbersalem.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>View Service</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>contact@apexplumbersalem.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(503) 974-3329</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>emergency plumber Salem OR</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:09 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3013,6 +3013,66 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Alliance Heating &amp; Air Conditioning | Antelope Valley HVAC Experts</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>callallianceac.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://callallianceac.com/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Improve Air</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>palmdaleallianceac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>661-992-2282</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>heating and cooling company Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:11 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3073,6 +3073,66 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Smith Roofing</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>smithroofingremodeling.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.smithroofingremodeling.com/residential-roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Jesse Smith</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>info@smithroofingremodeling.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(260) 577-8522</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>roof replacement Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:19 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3133,6 +3133,66 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>User's blog</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>billsroofinginc.net</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://billsroofinginc.net/service-areas/olympia/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Lake Gig</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>billsroofing@comcast.net</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>253-846-0833</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Olympia WA</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>residential roofing company Olympia WA</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:21 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3193,6 +3193,62 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>National Roofing</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>nationalroofing.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://nationalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@nationalroofing.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>505-883-3000</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>86</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>roofer Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:32 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3214,7 +3214,6 @@
           <t>https://nationalroofing.com/</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>info@nationalroofing.com</t>
@@ -3244,6 +3243,58 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Winter's Heating &amp; Air Conditoning | Lancaster, PA | York, PA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>wintersheatair.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://wintersheatair.com/york-pa/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>info@wintersheatair.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>86</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>heating and cooling company York PA</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:34 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3269,13 +3269,11 @@
           <t>https://wintersheatair.com/york-pa/</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>info@wintersheatair.com</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>York PA</t>
@@ -3295,6 +3293,66 @@
         </is>
       </c>
       <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Tackett Roofing</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>tackettroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://tackettroofingtx.com/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Roofing About</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@tackettroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(210) 761-7663</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>100</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>residential roofing company San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:38 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3358,6 +3358,126 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Happy Homesllp</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>happyhomesllp.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://happyhomesllp.com/roofing-services/las-cruces-nm/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>New Mexico</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>terroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(505) 382-4757</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>100</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>residential roofing company Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Roofing &amp; Stucco in Las Cruces, NM</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>gilbertandsonsroofingandstucco.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://gilbertandsonsroofingandstucco.com/service-areas/las-cruces</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>President Bob</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>gilbertandsons2010@gmail.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>575-649-2316</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>90</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>residential roofing company Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:43 UTC (cycle 175)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3478,6 +3478,66 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Roofing in Saint Charles, MO | iRestore STL</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>irestorestl.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://irestorestl.com/roofing/saint-charles-mo/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>By The</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>support@irestorestl.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(618) 641-9533</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>roof replacement St Charles MO</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:53 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3538,6 +3538,66 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>HomeServe of New England</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>homeservene.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.homeservene.com/locations/cambridge-ma/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Why Cambridge</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>david.johnson@strategicamerica.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(855) 288-8743</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Cambridge MA</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>100</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>heating and cooling company Cambridge MA</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 17:59 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3598,6 +3598,126 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Coral Springs Roofing Company | Repair &amp; Replacement | Free Quote</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>coconutcreekroofing.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.coconutcreekroofing.com/areas/coral-springs</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Coconut Creek</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>coconutcreekroofingfl@gmail.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(754) 307-7534</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>100</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>roof repair company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Boss Roofing</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>boss-roofing.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://boss-roofing.com/service-areas/broward/coral-springs/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>boss@boss-roofing.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(561) 766-3833</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>roof repair company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:00 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3718,6 +3718,126 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Rite Temp HVAC LLC</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ritetempnyc.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://ritetempnyc.com/hvac-services-queens/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Fully Insured</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>info@ritetempnyc.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>914-352-4822</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>100</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>heating and cooling company Queens NY</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Energo</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>energo.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://energo.com/hvac-services-in-queens/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>sales@energo.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>888.378.9898</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>98</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>heating and cooling company Queens NY</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:02 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3838,6 +3838,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Home | americanplumbing.pro</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>americanplumbing.pro</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://americanplumbing.pro/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Why Lansing</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>amy@americanplumbing.pro</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(517) 485-5550</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>88</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>plumbing company Lansing MI</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:03 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3898,6 +3898,62 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>365HeatingAndCooling</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>365heatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.365heatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>365cooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>435-922-5518</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>90</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>heating and cooling company St George UT</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:09 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3919,7 +3919,6 @@
           <t>https://www.365heatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>365cooling@gmail.com</t>
@@ -3949,6 +3948,66 @@
         </is>
       </c>
       <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Alpharetta, GA - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>hvacproalpharetta.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.hvacproalpharetta.com/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Rucker Rd</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>info@hvacproalpharetta.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(678) 264-6836</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>100</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>HVAC contractor Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:17 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4013,6 +4013,62 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Rapid City HVAC Services | Buzz's Heating and Cooling LLC</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>buzzshvac.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://buzzshvac.com/service-areas/rapid-city-sd</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>buzzsheatingandcooling@outlook.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>6054313675</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Rapid City SD</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>heating and cooling company Rapid City SD</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:24 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4034,7 +4034,6 @@
           <t>https://buzzshvac.com/service-areas/rapid-city-sd</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>buzzsheatingandcooling@outlook.com</t>
@@ -4064,6 +4063,126 @@
         </is>
       </c>
       <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Alpharetta</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>mayhvacga.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://mayhvacga.com/locations/alpharetta-ga/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Fast Estimates</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>info@mayhvacga.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(844) 606-1440</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>90</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>heat pump installation Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Repair in Alpharetta, GA</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>alpharetta-ga.ezhvacservices.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://alpharetta-ga.ezhvacservices.com/heat-pump-installation-repair/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>contact@ezhvacservices.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(833) 435-6630</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>heat pump installation Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:25 UTC (cycle 204)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4188,6 +4188,62 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Blair Plumbing - Plumber New Orleans</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>blairplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://blairplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@blairplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(504) 733-9113</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>90</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>plumber New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 18:27 UTC (cycle 205)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4209,7 +4209,6 @@
           <t>https://blairplumbinginc.com/</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>info@blairplumbinginc.com</t>
@@ -4239,6 +4238,62 @@
         </is>
       </c>
       <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Kellum Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>kellumroofing.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.kellumroofing.com/areas/glendale</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>jeremy@kellumroofing.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(480) 258-0925</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Glendale AZ</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>100</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>roof repair company Glendale AZ</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 19:56 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4264,7 +4264,6 @@
           <t>https://www.kellumroofing.com/areas/glendale</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>jeremy@kellumroofing.com</t>
@@ -4294,6 +4293,66 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>calvaryroofings</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>calvaryroofings.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://calvaryroofings.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Why Property</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>calvaryroofingsolutions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(475) 384-4225</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Waterbury CT</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>roofing contractor Waterbury CT</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:06 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4358,6 +4358,62 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Residential Roofing in Boise, ID | Martinez Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>martinezroofingid.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://martinezroofingid.com/home</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>example@eom.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(208) 906-6649</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>80</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>residential roofing company Boise ID</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:22 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4379,7 +4379,6 @@
           <t>https://martinezroofingid.com/home</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>example@eom.com</t>
@@ -4409,6 +4408,66 @@
         </is>
       </c>
       <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Water Heater Repair and Installation in Tampa, FL | Mr Water Heater</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>mrwaterheaterfl.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.mrwaterheaterfl.com/tampa/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Operated Tampa</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>mark@mrwaterheaterfl.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>727 203 8201</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>90</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>water heater repair Tampa FL</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:23 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4473,6 +4473,62 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Jack the Roofer Inc.</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>jacktherooferaz.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.jacktherooferaz.com/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>jack@jacktherooferaz.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(602) 975-3363</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>100</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>roofer Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:31 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4494,7 +4494,6 @@
           <t>https://www.jacktherooferaz.com/</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>jack@jacktherooferaz.com</t>
@@ -4524,6 +4523,66 @@
         </is>
       </c>
       <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>MGAH Construction</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>mgahnwa.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://www.mgahnwa.com/services/roofing</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Northwest Arkansas</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>mgahcons01@gmail.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(479) 419-0947</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Springdale AR</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Springdale AR</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:36 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4588,6 +4588,62 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Craftsman</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>craftsmanelectric.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.craftsmanelectric.com/covington-electrician-hvac-repair/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>info@craftsmanelectric.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>513-891-4426</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Covington KY</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>furnace repair Covington KY</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:38 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4609,7 +4609,6 @@
           <t>https://www.craftsmanelectric.com/covington-electrician-hvac-repair/</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>info@craftsmanelectric.com</t>
@@ -4639,6 +4638,66 @@
         </is>
       </c>
       <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Garland Roofing</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>metroplexflatmetal.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://metroplexflatmetal.com/garland-roofing/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>info@metroplexflatmetal.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(469) 600-0331</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Garland TX</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:42 UTC (cycle 33)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4703,6 +4703,62 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Comfort 360</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>mycomfort360.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://mycomfort360.com/air-conditioning-installation-gresham-or/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>info@comfortairnow.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(360) 891-2665</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Gresham OR</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>AC installation Gresham OR</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 20:45 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4724,7 +4724,6 @@
           <t>https://mycomfort360.com/air-conditioning-installation-gresham-or/</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>info@comfortairnow.com</t>
@@ -4754,6 +4753,66 @@
         </is>
       </c>
       <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>RAINDROP ROOFING NW | PORTLAND, OR</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>raindropnw.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.raindropnw.com/locations/hillsboro-or/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Roof Types</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>info@raindropnw.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(503)526-3887</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>90</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>residential roofing company Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:01 UTC (cycle 46)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4818,6 +4818,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Dreamstyle Roofing</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>dreamstyleroofing.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://dreamstyleroofing.com/residential-roofing-rio-rancho/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Submit Do</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>opt-out@dreamstyleus.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(505) 375-1619</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>residential roofing company Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:04 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4878,6 +4878,66 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Stars and Stripes Plumbing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>starsandstripesplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.starsandstripesplumbingco.com/moreno-valley-ca/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Stripes Plumbing</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>starsandstripesplumbingco@gmail.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>951-732-4194</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Moreno Valley CA</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>plumbing company Moreno Valley CA</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:06 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4938,6 +4938,126 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>jbroofing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>jbroofing.co</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://jbroofing.co/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Commercial Flat</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>info@jbroofing.co</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>402-939-6921</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>100</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>roofing contractor Omaha NE</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Priority Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>priorityplumbingri.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://priorityplumbingri.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Master Plumber</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>michaelcambio@priorityplumbing.net</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(401) 739-3700</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Warwick RI</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>98</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>plumbing company Warwick RI</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:07 UTC (cycle 50)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5058,6 +5058,62 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Plumbologyky2025</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>plumbologyky.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.plumbologyky.com/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>plumbing@plumbologyky.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>859-452-9963</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>90</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>plumber Lexington KY</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:12 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5079,7 +5079,6 @@
           <t>https://www.plumbologyky.com/</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>plumbing@plumbologyky.com</t>
@@ -5109,6 +5108,122 @@
         </is>
       </c>
       <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Archuleta Sewer &amp; Camera LLC | Cheyenne, WY</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>archuletasewer.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.archuletasewer.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>archuleta.sewer.camera@gmail.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(307) 287-4500</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>90</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>sewer repair Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Ekehoe</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>kehoeroofing.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://kehoeroofing.com/roof-replacement-san-diego/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>evan@kehoeroofing.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>858-395-5237</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>78</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>roof replacement San Diego CA</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:13 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5134,7 +5134,6 @@
           <t>https://www.archuletasewer.com/</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>archuleta.sewer.camera@gmail.com</t>
@@ -5224,6 +5223,126 @@
         </is>
       </c>
       <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Fort Worth, TX | Rockwater Plumbing</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>callrockwaterplumbing.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://www.callrockwaterplumbing.com/services/water-heater-repair-fort-worth-tx</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Reliable Water</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>rockwaterplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>817-659-5929</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>100</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>water heater repair Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Trusted Roofer in Independence, MO | Roof Angels</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>independence-mo.roofangels.org</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://independence-mo.roofangels.org/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Why Independence</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>info@roofangels.org</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(877) 510-0035</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Independence MO</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>80</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>roof replacement Independence MO</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:16 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5348,6 +5348,62 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Beauvais Plumbing Co.</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>beauvaisplumbingcollc.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.beauvaisplumbingcollc.com/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>support@webador.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>828-458-4611</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>74</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>plumbing company Asheville NC</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:22 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5369,7 +5369,6 @@
           <t>https://www.beauvaisplumbingcollc.com/</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>support@webador.com</t>
@@ -5399,6 +5398,62 @@
         </is>
       </c>
       <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Melton’s Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>meltonheating.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.meltonheating.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>info@meltonsheating.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>503.378.7482</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>90</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>air conditioning repair Salem OR</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:24 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5424,7 +5424,6 @@
           <t>https://www.meltonheating.com/</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>info@meltonsheating.com</t>
@@ -5454,6 +5453,66 @@
         </is>
       </c>
       <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Obsidian Roofing - Central Oregon</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>obsidian-roofing.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.obsidian-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Central Oregon</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>obsidianroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(541) 221-2118</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>88</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>roof replacement Bend OR</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:29 UTC (cycle 65)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5518,6 +5518,66 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Roofing Contractors Gainesville, FL | Florida Roof Masters</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>floridaroofmastersllc.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://floridaroofmastersllc.com/areas-served/gainesville-fl</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Mark Robertson</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>info@floridaroofmastersllc.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(352) 246-4980</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>88</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:41 UTC (cycle 73)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5578,6 +5578,118 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Certified Roof &amp; Inspection</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>roofcertified.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.roofcertified.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>ron@roofcertified.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(209) 252-0044</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>100</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>roof replacement Stockton CA</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Complete Crown Construction</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>completecrownconstruction.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://completecrownconstruction.com/services/metal-roofing/abilene</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>completecrownconstruction@gmail.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(254) 246-2966</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>88</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Abilene TX</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:42 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5599,7 +5599,6 @@
           <t>https://www.roofcertified.com/</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>ron@roofcertified.com</t>
@@ -5655,7 +5654,6 @@
           <t>https://completecrownconstruction.com/services/metal-roofing/abilene</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>completecrownconstruction@gmail.com</t>
@@ -5685,6 +5683,122 @@
         </is>
       </c>
       <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Heat Pump Replacement in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.mayflowerhvac.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.mayflowerhvac.com/heat-pump-replacement/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Cleaning Furnace</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>contact@mayflowerhvac.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(833) 959-4477</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>heat pump installation Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Heat Pump Replacement in Aberdeen, SD | Fully Licensed HVAC Service</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.dougshvacllc.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.dougshvacllc.com/heat-pump-replacement/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>contact@dougshvacllc.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(833) 959-4477</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>90</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>heat pump installation Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 21:47 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5769,7 +5769,6 @@
           <t>https://aberdeen-sd.dougshvacllc.com/heat-pump-replacement/</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>contact@dougshvacllc.com</t>
@@ -5799,6 +5798,62 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Air Conditioning Company Augusta, GA</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>allweatherga.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.allweatherga.com/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>allweatherhvacga@gmail.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(706) 237-2377</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Augusta GA</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>100</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>heating and cooling company Augusta GA</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:01 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5824,7 +5824,6 @@
           <t>https://www.allweatherga.com/</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>allweatherhvacga@gmail.com</t>
@@ -5854,6 +5853,126 @@
         </is>
       </c>
       <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Find a HVAC Pro | Mitsubishi Electric HVAC US</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>mitsubishicomfort.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.mitsubishicomfort.com/find-pros</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Andrew Kelso</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>customercare@hvac.mea.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(800) 433-4822</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>heat pump installation Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Bosch Home Comfort</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>bosch-homecomfort.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.bosch-homecomfort.com/us/en/residential/service-support/installer-locator/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Bulletins Overview</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>privacy.policy@us.bosch.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>6144124545</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>86</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>heat pump installation Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:13 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5978,6 +5978,62 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Carolina Boys Plumbing</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>cboysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://cboysplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>sirtony813@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(803) 479-9190</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>90</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>plumbing company Columbia SC</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:16 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5999,7 +5999,6 @@
           <t>https://cboysplumbing.com/</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>sirtony813@yahoo.com</t>
@@ -6029,6 +6028,66 @@
         </is>
       </c>
       <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>A&amp;S Plumbing | Plumbers in Louisville Ky</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>asplumbingcompany.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.asplumbingcompany.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Kitchen Faucet</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>aandsplumber@gmail.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(502) 451-4955</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>100</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>plumber Louisville KY</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:29 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6093,6 +6093,126 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Plumbing contractors</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>minneapolismn.gov</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.minneapolismn.gov/business-services/licenses-permits-inspections/business-licenses/contractors/licensed-contractors/plumbing/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Property Information</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>minneapolis311@minneapolismn.gov</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>612-673-3000</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>plumbing company Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Pipe Dream Plumbing Co.</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>pipedreamplumbersca.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.pipedreamplumbersca.com/locations/escondido/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Dream Plumbing</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>office@pipedreamplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(858) 330-2881</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>90</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>plumbing company Escondido CA</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:30 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6213,6 +6213,66 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>TheRoofingBrief</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>theroofingbrief.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://theroofingbrief.com/best-roofers-brownsville-tx/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Subscribe Roofing</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>info@theroofingbrief.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(956) 546-6638</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Brownsville TX</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>100</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>roof replacement Brownsville TX</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:43 UTC (cycle 116)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6273,6 +6273,66 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Guns N Hoses Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>gunsnhosesllc.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://gunsnhosesllc.com/roofing-grand-rapids-mi/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Hoses Roofing</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>gnhroofs@gmail.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(810) 226-0400</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>residential roofing company Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:48 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6333,6 +6333,62 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>One &amp; Done Roofing</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>rochesterasphaltroofing.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://rochesterasphaltroofing.com/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>oneanddonebuildersllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(585) 455-2459</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>100</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>roofing contractor Rochester NY</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:49 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6354,7 +6354,6 @@
           <t>https://rochesterasphaltroofing.com/</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>oneanddonebuildersllc@gmail.com</t>
@@ -6384,6 +6383,66 @@
         </is>
       </c>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Sewer Line Repairs Broken Arrow, OK | Cooper Perry Plumbing</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>cooperperryplumbing.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.cooperperryplumbing.com/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Signs You</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>cpplumbingtulsa@gmail.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(918) 328-0009</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>sewer repair Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:52 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6448,6 +6448,66 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Heating &amp; Cooling in Concord, NC | Peaks Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>peaksheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://peaksheatingandcooling.com/service-areas/concord</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Based In</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>peaksheatingcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(704) 452-4893</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>100</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>heating and cooling company Concord NC</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 22:54 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6508,6 +6508,62 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>AC Repair In Richardson</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>acrepairinrichardson.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://acrepairinrichardson.com/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>contact@acrepairinrichardson.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(817) 670-8692</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>100</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>air conditioning repair Richardson TX</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:00 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6529,7 +6529,6 @@
           <t>https://acrepairinrichardson.com/</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>contact@acrepairinrichardson.com</t>
@@ -6559,6 +6558,126 @@
         </is>
       </c>
       <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Assured Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>assuredheatcool.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://assuredheatcool.com/cooling/installation-replacement/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>At Assured</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>info@assuredheatcool.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>314-651-5969</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>88</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>AC installation St Louis MO</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Johns Drains</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>johnsdrains.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://johnsdrains.com/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Video Inspection</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>info@johnsdrains.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(612) 756-7394</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>80</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>drain cleaning service Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:14 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6683,6 +6683,62 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>My AC Guy</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>myacserviceguy.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.myacserviceguy.com/furnace-and-heat-pump-installation-and-replacement-services/lakeland</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>scottcorley1985@gmail.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>813-541-5642</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>84</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>heat pump installation Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:19 UTC (cycle 140)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6704,7 +6704,6 @@
           <t>https://www.myacserviceguy.com/furnace-and-heat-pump-installation-and-replacement-services/lakeland</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>scottcorley1985@gmail.com</t>
@@ -6734,6 +6733,126 @@
         </is>
       </c>
       <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Brehm Roofing - Gainesville FL Roofing Professionals</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>brehmroofing.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://brehmroofing.com/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Blog Contact</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@brehmroofing.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>352-664-8585</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>100</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>roofer Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Duffield Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>duffieldroofingandexteriors.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://duffieldroofingandexteriors.com/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>email@emailaddress.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(352) 375-7008</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>100</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>roofer Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:22 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6858,6 +6858,62 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Northwind Heat And Air, Inc.</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>northwindheatandair.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.northwindheatandair.com/norman-ok-heating-air-conditioning-contractor/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>ranaewinterton@gmail.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>405-527-7135</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Norman OK</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>100</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>heating and cooling company Norman OK</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:23 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6879,7 +6879,6 @@
           <t>https://www.northwindheatandair.com/norman-ok-heating-air-conditioning-contractor/</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>ranaewinterton@gmail.com</t>
@@ -6909,6 +6908,66 @@
         </is>
       </c>
       <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Cheyenne, WY Roofing Services | Trusted Roof Solutions | Roof Check Inc</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>roof-check.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://roof-check.com/service-areas/cheyenne-wy</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Downspouts Protect</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>info@roof-check.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>8657375043</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>roof repair company Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:25 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6973,6 +6973,66 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Man of Steel Roofer of Lawrence KS</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>lawrenceroofer.manofsteelresources.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://lawrenceroofer.manofsteelresources.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@lawrenceroofer.manofsteelresources.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(785) 330-5727</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Lawrence KS</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>90</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roofing contractor Lawrence KS</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:29 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7033,6 +7033,62 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Metal Roofing Mesquite</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>rowesroofing.net</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://rowesroofing.net/areas-of-service/mesquite-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>steverowe@rocketmail.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>(972) 276-1978</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Mesquite TX</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>100</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Mesquite TX</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:35 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7054,7 +7054,6 @@
           <t>https://rowesroofing.net/areas-of-service/mesquite-metal-roofing/</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>steverowe@rocketmail.com</t>
@@ -7084,6 +7083,66 @@
         </is>
       </c>
       <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Furnace Repair in Pompano Beach, FL | Same-Day Service</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>usafirstac.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.usafirstac.com/services/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Pompano Beach</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>info@usafirstac.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(561) 473-4178</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Pompano Beach FL</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>84</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>furnace repair Pompano Beach FL</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:36 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7148,6 +7148,66 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>AJ Danboise – Plumbing, Heating, Cooling &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ajdanboise.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://ajdanboise.com/service-areas/livonia-mi/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Ream More</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>info@ajdanboise.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(248) 236-5999</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Livonia MI</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>AC installation Livonia MI</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:39 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7208,6 +7208,126 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>H. Hulse Heating</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>hhulse.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://www.hhulse.com/areas-we-serve/hvac-stamford-ct/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Hulse Heating</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>office@hhulse.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>(203) 380 2692</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>100</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>heating and cooling company Stamford CT</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Roofing Company in Birmingham</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>alabamaroofrx.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://alabamaroofrx.com/service-category/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>You Can</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>alroofrx@gmail.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(205) 649-4950</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>88</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>residential roofing company Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:46 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7328,6 +7328,66 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Roofing Technologies Unlimited</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>roofingtechnologiesunlimitedtx.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://roofingtechnologiesunlimitedtx.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Why Katy</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>info@rtuhtx.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(832) 866-9595</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>residential roofing company Katy TX</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:48 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7388,6 +7388,66 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>General Mechanix</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>generalmechanix.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://generalmechanix.com/hvac-services-bangor-maine/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Services About</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>info@generalmechanix.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>207-951-0817</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Bangor ME</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>84</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>HVAC contractor Bangor ME</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:51 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7448,6 +7448,66 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>BEST Plumbers in Laramie, WY - Sunshine Plumbers</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>sunshine-plumbers.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.sunshine-plumbers.com/location/laramie-wy</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Sunshine Plumbers</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>info@sunshine-plumbers.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(844) 822-7445</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Laramie WY</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>plumbing company Laramie WY</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-25 23:58 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-25.xlsx
+++ b/output/leads_2026-09-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7508,6 +7508,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Ralph’s Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>ralphsroofing.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://ralphsroofing.com/metal-roofing-baton-rouge</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Now Get</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>info@ralphsroofing.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(225) 610-4116</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>100</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>